<commit_message>
chek in para que blas lo clone
</commit_message>
<xml_diff>
--- a/Automation Anywhere/Bots/TrivalentePolizas/Docs/Catalogos.xlsx
+++ b/Automation Anywhere/Bots/TrivalentePolizas/Docs/Catalogos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emergys1-my.sharepoint.com/personal/hector_agraz_emergys_com/Documents/PoC/trivalente/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="11_F25DC773A252ABDACC104837715E4E725BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B269C304-3304-48A8-B5EA-35E86930DE43}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="11_F25DC773A252ABDACC104837715E4E725BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96143EC7-BEA0-4AB7-8B52-6E9F92411D5A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Key</t>
   </si>
@@ -48,18 +48,9 @@
     <t>GetComp</t>
   </si>
   <si>
-    <t>Obtener el listado de las empresas a diccionario</t>
-  </si>
-  <si>
     <t>LoginXML</t>
   </si>
   <si>
-    <t>Company</t>
-  </si>
-  <si>
-    <t>Empresa: {0}</t>
-  </si>
-  <si>
     <t>Ingresando al Aplicativo Descarga y administración Masiva de XML</t>
   </si>
   <si>
@@ -67,6 +58,87 @@
   </si>
   <si>
     <t>CloseXML</t>
+  </si>
+  <si>
+    <t>ErrorXML</t>
+  </si>
+  <si>
+    <t>LoginContpaqi</t>
+  </si>
+  <si>
+    <t>CloseContpaqi</t>
+  </si>
+  <si>
+    <t>Ingresando al Aplicativo Contpaqi</t>
+  </si>
+  <si>
+    <t>Cerrando Contpaqi</t>
+  </si>
+  <si>
+    <t>No se pudo abrir Contpaqi</t>
+  </si>
+  <si>
+    <t>No se pudo abrir Descarga y administración Masiva de XML</t>
+  </si>
+  <si>
+    <t>ErrorContpaqi</t>
+  </si>
+  <si>
+    <t>ErrorEmpresa</t>
+  </si>
+  <si>
+    <t>RFC De Empresa: {0}</t>
+  </si>
+  <si>
+    <t>No se pudo encontrar la empresa {0} en ContPaqi</t>
+  </si>
+  <si>
+    <t>LoadingEmitted</t>
+  </si>
+  <si>
+    <t>Empezando con la carga de XMLs emitidos</t>
+  </si>
+  <si>
+    <t>EnterPath</t>
+  </si>
+  <si>
+    <t>Ingresando ruta para abrir carpeta de XML{0}</t>
+  </si>
+  <si>
+    <t>LoadXMLs</t>
+  </si>
+  <si>
+    <t>CargandoXMLs</t>
+  </si>
+  <si>
+    <t>CompanyRFC</t>
+  </si>
+  <si>
+    <t>CompanyName</t>
+  </si>
+  <si>
+    <t>Nombre de la empresa: {0}</t>
+  </si>
+  <si>
+    <t>GetCompanyRFC</t>
+  </si>
+  <si>
+    <t>Obtener lista de RFC de empresas a diccionaroo</t>
+  </si>
+  <si>
+    <t>Obtener listado de nombre de empresas a diccionario</t>
+  </si>
+  <si>
+    <t>NoConsolidarte</t>
+  </si>
+  <si>
+    <t>No se encontro el archivo consolidado</t>
+  </si>
+  <si>
+    <t>Archivo validar {0}</t>
+  </si>
+  <si>
+    <t>SearhConsolidate</t>
   </si>
 </sst>
 </file>
@@ -429,13 +501,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -443,7 +516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -451,7 +524,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -459,64 +532,154 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
         <v>9</v>
       </c>
-      <c r="B5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="K13" s="3"/>
-    </row>
-    <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="K14" s="3"/>
-    </row>
-    <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="K15" s="3"/>
-    </row>
-    <row r="16" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="K16" s="3"/>
-    </row>
-    <row r="17" spans="11:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" t="s">
+        <v>23</v>
+      </c>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" spans="11:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" t="s">
+        <v>25</v>
+      </c>
       <c r="K18" s="3"/>
     </row>
-    <row r="19" spans="11:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="K19" s="4"/>
-    </row>
-    <row r="20" spans="11:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" t="s">
+        <v>27</v>
+      </c>
+      <c r="K19" s="3"/>
+    </row>
+    <row r="20" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="K20" s="3"/>
     </row>
-    <row r="22" spans="11:11" x14ac:dyDescent="0.25">
-      <c r="K22" s="5"/>
+    <row r="21" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="K22" s="3"/>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="K23" s="4"/>
+    </row>
+    <row r="24" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="K24" s="3"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K26" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>